<commit_message>
Fixed issues. Code notebooks into CODE folder.
</commit_message>
<xml_diff>
--- a/CLEANED DATA/REMX.K-USD-clean.xlsx
+++ b/CLEANED DATA/REMX.K-USD-clean.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REMX_clean" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="REMX_clean" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11380,7 +11380,7 @@
         <v>6.391859626458581e-05</v>
       </c>
       <c r="I377" t="n">
-        <v>7.598454826554365e-05</v>
+        <v>7.598454826554364e-05</v>
       </c>
     </row>
     <row r="378">
@@ -40380,7 +40380,7 @@
         <v>5.414174289552053e-05</v>
       </c>
       <c r="I1377" t="n">
-        <v>7.704862662897478e-05</v>
+        <v>7.704862662897477e-05</v>
       </c>
     </row>
     <row r="1378">

</xml_diff>